<commit_message>
more datacamp and disk_savvy data
</commit_message>
<xml_diff>
--- a/datacamp.xlsx
+++ b/datacamp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\NAUKA\Python Nauka\data_science\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747E5906-1162-4E70-931D-ED36ABF02F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB71310-4708-4B12-9E7D-5325EEA85019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5355" yWindow="5355" windowWidth="5070" windowHeight="9375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5700" yWindow="5700" windowWidth="5070" windowHeight="9375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -205,12 +205,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="406" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="407" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3473,11 +3481,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="407">
+  <cellXfs count="408">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="403" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="402" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="404" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="401" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="403" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="400" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="399" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="398" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3493,10 +3502,10 @@
     <xf numFmtId="0" fontId="388" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="387" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="386" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="385" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="403" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="404" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="385" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="384" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="383" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="382" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3756,9 +3765,9 @@
     <xf numFmtId="0" fontId="128" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="127" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="126" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="405" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="406" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="125" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="404" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="405" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="124" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="123" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="122" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6144,7 +6153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
         <v>28</v>
       </c>
@@ -6205,8 +6214,11 @@
       <c r="T33" s="371">
         <v>5</v>
       </c>
+      <c r="U33" s="407">
+        <v>3</v>
+      </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>29</v>
       </c>
@@ -6268,7 +6280,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>30</v>
       </c>
@@ -6330,7 +6342,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>31</v>
       </c>
@@ -6392,7 +6404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>35</v>
       </c>
@@ -6452,7 +6464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>32</v>
       </c>
@@ -6514,7 +6526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>42</v>
       </c>
@@ -6561,7 +6573,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>36</v>
       </c>
@@ -6611,7 +6623,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>37</v>
       </c>
@@ -6661,7 +6673,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>44</v>
       </c>
@@ -6702,7 +6714,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>45</v>
       </c>
@@ -6743,7 +6755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>46</v>
       </c>
@@ -6784,7 +6796,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>47</v>
       </c>
@@ -6825,7 +6837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>48</v>
       </c>
@@ -6866,7 +6878,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>51</v>
       </c>
@@ -6902,7 +6914,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>52</v>
       </c>

</xml_diff>